<commit_message>
Refine Angélica's brief template and instructions, updating the Excel format to enhance clarity and usability. Adjust CSV content to provide more descriptive text for each entry, ensuring accurate representation of visual elements. Update the script to accommodate new formatting and improve user guidance on filling out the brief, emphasizing the handling of overlapping images. Enhance documentation to reflect these changes and streamline the workflow for generating engine-ready YAML.
</commit_message>
<xml_diff>
--- a/templates/angelica_brief/plantilla_reel_angelica.xlsx
+++ b/templates/angelica_brief/plantilla_reel_angelica.xlsx
@@ -441,15 +441,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -480,10 +478,10 @@
       </c>
       <c r="B3" t="inlineStr"/>
     </row>
-    <row r="4" ht="36" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Tiempos = TU video original (no Instagram). Pega la foto en Foto. Lado: derecha, izquierda o arriba. Sin foto = título en el cielo (escribe Texto). La tarjeta de WhatsApp del final se pone sola.</t>
+          <t>Escribe con tus palabras. Reloj = TU video, no Instagram. Pega la foto en Foto. En «Qué quieres» di qué se ve y dónde (derecha / izquierda / arriba). Si dos fotos se ven juntas, son dos filas. Cursor arma el reel.</t>
         </is>
       </c>
     </row>
@@ -505,80 +503,77 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Texto</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Lado</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Nota</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="64" customHeight="1">
+          <t>Qué quieres</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="88" customHeight="1">
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="n"/>
-    </row>
-    <row r="8" ht="64" customHeight="1">
+      <c r="D7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="88" customHeight="1">
       <c r="A8" s="4" t="n"/>
       <c r="B8" s="4" t="n"/>
-    </row>
-    <row r="9" ht="64" customHeight="1">
+      <c r="D8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="88" customHeight="1">
       <c r="A9" s="4" t="n"/>
       <c r="B9" s="4" t="n"/>
-    </row>
-    <row r="10" ht="64" customHeight="1">
+      <c r="D9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="88" customHeight="1">
       <c r="A10" s="4" t="n"/>
       <c r="B10" s="4" t="n"/>
-    </row>
-    <row r="11" ht="64" customHeight="1">
+      <c r="D10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="88" customHeight="1">
       <c r="A11" s="4" t="n"/>
       <c r="B11" s="4" t="n"/>
-    </row>
-    <row r="12" ht="64" customHeight="1">
+      <c r="D11" s="4" t="n"/>
+    </row>
+    <row r="12" ht="88" customHeight="1">
       <c r="A12" s="4" t="n"/>
       <c r="B12" s="4" t="n"/>
-    </row>
-    <row r="13" ht="64" customHeight="1">
+      <c r="D12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="88" customHeight="1">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="n"/>
-    </row>
-    <row r="14" ht="64" customHeight="1">
+      <c r="D13" s="4" t="n"/>
+    </row>
+    <row r="14" ht="88" customHeight="1">
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="64" customHeight="1">
+      <c r="D14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="88" customHeight="1">
       <c r="A15" s="4" t="n"/>
       <c r="B15" s="4" t="n"/>
-    </row>
-    <row r="16" ht="64" customHeight="1">
+      <c r="D15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="88" customHeight="1">
       <c r="A16" s="4" t="n"/>
       <c r="B16" s="4" t="n"/>
-    </row>
-    <row r="17" ht="64" customHeight="1">
+      <c r="D16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="88" customHeight="1">
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="n"/>
-    </row>
-    <row r="18" ht="64" customHeight="1">
+      <c r="D17" s="4" t="n"/>
+    </row>
+    <row r="18" ht="88" customHeight="1">
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="E7:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" prompt="derecha / izquierda de la cabeza, o arriba (título)" type="list">
-      <formula1>"derecha,izquierda,arriba"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>